<commit_message>
fix: faster cable disconnect detection, Excel report tab names, remove Word/PDF
Cable detection:
- Reduce FAIL_THRESHOLD from 3 to 2 and PING_INTERVAL from 3s to 2s
  for faster disconnect detection (4s instead of 9s)
- Reduce TCP probe timeout from 3s to 2s
- Add pre-test connectivity check before each test starts — catches
  disconnects that happened between monitor poll intervals
- If pre-test probe fails, waits for cable handler to pause before
  retrying

Report format:
- Rename Excel template tabs: TEST SUMMARY -> General Test Information,
  TESTPLAN -> Test Results, ADDITIONAL INFORMATION -> Additional Device
  Information (matches Electracom qualification template)
- Update generic.json cell mapping to match new tab names
- Remove Word and PDF from report format options (Excel only)

Co-Authored-By: claude-flow <ruv@ruv.net>
</commit_message>
<xml_diff>
--- a/templates/[MANUFACTURER] - [MODEL] - IP Device Qualification Template (Rev00) C00.xlsx
+++ b/templates/[MANUFACTURER] - [MODEL] - IP Device Qualification Template (Rev00) C00.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:ns5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:ns6="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:ns8="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:ns9="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29917"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ecprojects.sharepoint.com/sites/MSITeam/Shared Documents/Solutions &amp; Technical/Technical Templates/Device Qualification/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="462" documentId="8_{5318B0E2-893C-4AA4-B9FA-06DD98A5A517}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B1ADB3FC-BCDE-4EBC-B79B-2AAE33FD6864}"/>
+  <ns1:AlternateContent>
+    <ns1:Choice Requires="x15">
+      <ns2:absPath url="https://ecprojects.sharepoint.com/sites/MSITeam/Shared Documents/Solutions &amp; Technical/Technical Templates/Device Qualification/"/>
+    </ns1:Choice>
+  </ns1:AlternateContent>
+  <ns3:revisionPtr revIDLastSave="462" documentId="8_{5318B0E2-893C-4AA4-B9FA-06DD98A5A517}" ns4:coauthVersionLast="47" ns4:coauthVersionMax="47" ns5:uidLastSave="{B1ADB3FC-BCDE-4EBC-B79B-2AAE33FD6864}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="900" xr2:uid="{A2A9A283-2B35-4B28-B903-8DACAC418321}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="900" ns6:uid="{A2A9A283-2B35-4B28-B903-8DACAC418321}"/>
   </bookViews>
   <sheets>
-    <sheet name="TEST SUMMARY" sheetId="60" r:id="rId1"/>
-    <sheet name="TESTPLAN" sheetId="61" r:id="rId2"/>
-    <sheet name="ADDITIONAL INFORMATION" sheetId="62" r:id="rId3"/>
+    <sheet name="General Test Information" sheetId="60" r:id="rId1"/>
+    <sheet name="Test Results" sheetId="61" r:id="rId2"/>
+    <sheet name="Additional Device Information" sheetId="62" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">TESTPLAN!$B$10:$G$53</definedName>
@@ -25,19 +25,19 @@
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <ns8:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
+    <ext uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <ns9:calcFeatures>
+        <ns9:feature name="microsoft.com:RD"/>
+        <ns9:feature name="microsoft.com:Single"/>
+        <ns9:feature name="microsoft.com:FV"/>
+        <ns9:feature name="microsoft.com:CNMTM"/>
+        <ns9:feature name="microsoft.com:LET_WF"/>
+        <ns9:feature name="microsoft.com:LAMBDA_WF"/>
+        <ns9:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </ns9:calcFeatures>
     </ext>
   </extLst>
 </workbook>

</xml_diff>